<commit_message>
任务表: 1.3.6 压测 / 1.3.7 转接板真引脚 / 1.3.9 lane47 结论 / 1.3.14 UL_IDLE_OK 四项完成 (dr1v90 feature/lvds-b2b efbab52)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/验证板任务分解_2026-10-10.xlsx
+++ b/docs/验证板任务分解_2026-10-10.xlsx
@@ -12,7 +12,7 @@
     <sheet name="汇总" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任务分解'!$A$1:$M$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任务分解'!$A$1:$M$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1019,25 +1019,25 @@
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>本机 lz4 帧能翻页 → WiFi 收流; 连推 ≥200 帧不卡</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>本机 lz4 帧能翻页; 连推 ≥200 帧不卡</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>自测→合测</t>
+          <t>自测</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>DR1M90 (+屏)</t>
+          <t>DR1M90</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
@@ -1052,14 +1052,10 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>能编不能跑 (缺 povmem+显示 PL, 现已具备)</t>
-        </is>
-      </c>
-      <c r="M6" s="7" t="inlineStr">
-        <is>
-          <t>D6</t>
-        </is>
-      </c>
+          <t>D6 10-10 无人值守: CPU 400/400、PL 2000/2000 帧无回退无超时 (V90 第 37 帧卡死问题 M90 无); 工具 board/pvsplay (dr1v90 3357208)</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1076,16 +1072,16 @@
       <c r="D7" s="7" t="inlineStr"/>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>PVS1 / povsh; 静止台架 flip 稳定</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>🔶进行中</t>
+          <t>PVS1 / povstream; 静止台架 flip 稳定, 空闲动画让位</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
@@ -1094,7 +1090,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>DR1M90 + AP + PC</t>
+          <t>DR1M90 + 办公 WiFi undef + PC</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
@@ -1109,14 +1105,10 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>WiFi TCP 159 Mbps (project_dr1m90_wifi_retest)</t>
-        </is>
-      </c>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>D7</t>
-        </is>
-      </c>
+          <t>D7: 12 fps 600/600 帧 (PL), 发送 11.86 fps / 18 Mbps; 空闲动画让位/恢复正常</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -1127,22 +1119,22 @@
       <c r="B8" s="7" t="inlineStr"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>开机自启</t>
+          <t>开机自启 / 打包</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>povboot AUTOBOOT: 冷启动一次到可推流</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>povboot AUTOBOOT: 冷启动一次到可推流; 打包脚本按架构选</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>🔶进行中</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
@@ -1156,7 +1148,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>脚本改造可脱离</t>
+          <t>脚本已离线完成</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
@@ -1166,12 +1158,12 @@
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>7 处 _riscv64 写死清单 (D1 agent); 卡上已有 up.sh</t>
+          <t>tools/pov_arch.sh + 6 个脚本 aarch64 化, dry-run 两架构 PASS; povsh_aarch64 已出</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>D18; 打包脚本 aarch64 化可先做</t>
+          <t>D18: aarch64 rootfs (S95pov) + povboot 加载后写 0x33</t>
         </is>
       </c>
     </row>
@@ -1339,63 +1331,87 @@
       <c r="M11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>DR1M90 · PL 逻辑</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>显示/取片 (2047 回归) + lz4 + 上行发送 (→GW5A)</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>🔶进行中</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr"/>
-      <c r="K12" s="5" t="inlineStr"/>
-      <c r="L12" s="5" t="inlineStr"/>
-      <c r="M12" s="5" t="inlineStr"/>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>1.1.10</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr"/>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>板端体素→切片</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>切片放 A35 还是 PL: CPU 路径 DDR 占 83% (12 fps) / PL 直供 28%; 列中心半像素、面 B 相位只加一次、gamma/径向补偿</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>⬜未开始</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>自测</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>DR1M90</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>算法已离线对拍</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>agent C 10-10: vb_slice_all.c x86/aarch64 可编, 8 条板端待决问题见 project_host_validation_profile_358</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>D6/D16; 建议 PL 直供</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>1.2.1</t>
+          <t>1.1.11</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr"/>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>2047 显示位流 (M90)</t>
+          <t>远程升级 (X4)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr"/>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>构建 + 加载 + 上屏</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>🔶进行中</t>
+          <t>SD 卡 A/B 槽位; 热切换 + 自检窗口 + 自动回滚; 开机 trial 回退; GW5A 每次上电由 DR1 灌, 不写 Flash; 内核第一期不做</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>⬜未开始</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -1404,42 +1420,46 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>DR1M90 + 2047 屏</t>
+          <t>DR1M90 + WiFi (+ACG525 验 GW5A 灌)</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>构建可脱离</t>
+          <t>工具/脚本可脱离</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>D1 bin md5 2ac42cbb; D2 PASS</t>
-        </is>
-      </c>
-      <c r="M13" s="7" t="inlineStr"/>
+          <t>计划 §10 (10-10 用户定)</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>D18–D19 之后, ≈2.5 天</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>1.2.1.a</t>
+          <t>1.1.11.a</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr"/>
       <c r="C14" s="7" t="inlineStr"/>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>单面全白 (D4)</t>
+          <t>槽位 + MANIFEST + PC 推送工具</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>m90_firstlight.sh s1→s3, 不掉电</t>
+          <t>povota push 只写非当前槽, sha256 校验</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
@@ -1452,51 +1472,47 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>系统</t>
+          <t>自测</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>2047 屏 (焊接中)</t>
+          <t>DR1M90</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>大部分可</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="L14" s="7" t="inlineStr">
-        <is>
-          <t>脚本无屏空跑通过</t>
-        </is>
-      </c>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr"/>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>等屏</t>
+          <t>0.5 天</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>1.2.1.b</t>
+          <t>1.1.11.b</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr"/>
       <c r="C15" s="7" t="inlineStr"/>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>双面全白 (D5)</t>
+          <t>热切换 + 自检 + 自动回滚</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>dual_en, PHASE_B=180, mirror_a/b=0, 无花屏</t>
+          <t>GP0 MAGIC / link_up / 好帧计数 / PC 心跳</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -1509,12 +1525,12 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>系统</t>
+          <t>合测</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>2047 屏</t>
+          <t>DR1M90 + WiFi</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
@@ -1524,36 +1540,32 @@
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>脚本无屏空跑通过</t>
-        </is>
-      </c>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr"/>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>等屏</t>
+          <t>1 天</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>1.2.1.c</t>
+          <t>1.1.11.c</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr"/>
       <c r="C16" s="7" t="inlineStr"/>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>3-bit / 偏心几何 (D8/D9)</t>
+          <t>开机 trial 回退</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>棋盘/斜坡与 7020 同图; 转起来体像方向对</t>
+          <t>trial 未清 ⇒ 起旧槽位</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -1566,12 +1578,12 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>系统</t>
+          <t>自测</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>2047 屏 + 电机</t>
+          <t>DR1M90</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
@@ -1581,179 +1593,171 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="L16" s="7" t="inlineStr">
-        <is>
-          <t>cmds_3bit_working.txt (V90 09-01)</t>
-        </is>
-      </c>
-      <c r="M16" s="7" t="inlineStr"/>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr"/>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>0.5 天</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.1.11.d</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr"/>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>PL lz4 三引擎 (M90)</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr"/>
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>故障注入</t>
+        </is>
+      </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>解压正确 + 并发不扰取片</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+          <t>坏包 / 自检失败 / 切换中掉电 各 ≥5 次不变砖</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>⬜未开始</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>DR1M90 + WiFi</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>0.5 天</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>DR1M90 · PL 逻辑</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>显示/取片 (2047 回归) + lz4 + 上行发送 (→GW5A)</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>🔶进行中</t>
         </is>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G18" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>自测</t>
-        </is>
-      </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>DR1M90</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr"/>
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr"/>
+      <c r="M18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>1.2.1</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr"/>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>2047 显示位流 (M90)</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr"/>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>构建 + 加载 + 上屏</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>🔶进行中</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>自测→系统</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>DR1M90 + 2047 屏</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>构建可脱离</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="L17" s="7" t="inlineStr">
-        <is>
-          <t>D2 自检: NENG=3, 寄存器读写对</t>
-        </is>
-      </c>
-      <c r="M17" s="7" t="inlineStr">
-        <is>
-          <t>D10; 可先在板上单独验解压</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>1.2.3</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr"/>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>上行发送 uplink_tx (→GW5A)</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr"/>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>13 lane 真帧, 800M / 1.0G; M90 器件综合收敛</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>自测→合测</t>
-        </is>
-      </c>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>综合: 无; 合测: DR1M90+ACG525 飞线</t>
-        </is>
-      </c>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>综合可脱离</t>
-        </is>
-      </c>
-      <c r="K18" s="7" t="inlineStr">
-        <is>
-          <t>综合是</t>
-        </is>
-      </c>
-      <c r="L18" s="7" t="inlineStr">
-        <is>
-          <t>09-18 800M RTL 已有 (V90); 发端与 GW5A 收端 tb 对拍过</t>
-        </is>
-      </c>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>D12 综合; D13/X2 环回</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>1.3</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>GW5A-25 · 桥片固件</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr"/>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>上行接收 → 分发 → 2260 序列器 → tx 阵列; 两模式</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>🔶进行中</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="H19" s="5" t="inlineStr"/>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="5" t="inlineStr"/>
-      <c r="K19" s="5" t="inlineStr"/>
-      <c r="L19" s="5" t="inlineStr"/>
-      <c r="M19" s="5" t="inlineStr"/>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>D1 bin md5 2ac42cbb; D2 PASS</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>1.3.1</t>
+          <t>1.2.1.a</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr"/>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>上行接收 rtl_x8</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr"/>
+      <c r="C20" s="7" t="inlineStr"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>单面验证 (D4)</t>
+        </is>
+      </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>IDES8 + 对齐 + deskew</t>
+          <t>三色循环 + 数字棋盘格, 低亮度起 (用户定流程)</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1766,157 +1770,161 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>自测</t>
+          <t>系统</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>ACG525</t>
+          <t>2047 屏 (DR1M90-02)</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>仿真可</t>
+          <t>否</t>
         </is>
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>gw5a_loop 4lane@400M 硅上 0 错; bench 13 lane 片内</t>
-        </is>
-      </c>
-      <c r="M20" s="7" t="inlineStr">
-        <is>
-          <t>800M 长线待短绞线</t>
-        </is>
-      </c>
+          <t>10-10: Bank11 跳帽改 3.3V 后 s1 ✅ 三色循环 ✅ 数字棋盘格 ✅ (用户目视)</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>1.3.2</t>
+          <t>1.2.1.b</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr"/>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>分发 + 帧门控</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr"/>
+      <c r="C21" s="7" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>双面全白 (D5)</t>
+        </is>
+      </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>逐像素正确; 刷新不坏帧 (UL_DROP)</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>✅完成</t>
+          <t>dual_en, PHASE_B=180, mirror_a/b=0, 无花屏</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>🔶进行中</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>自测</t>
+          <t>系统</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>ACG525</t>
+          <t>2047 屏</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>仿真可</t>
+          <t>否</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>gw5a_bench 1025 万帧 0 坏, 0 retrain</t>
-        </is>
-      </c>
-      <c r="M21" s="7" t="inlineStr"/>
+          <t>10-10 双面电气通过 (engB_busy=1, duty 0.041, 10 s 不掉电); 用户外出, 目视待回来</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>目视</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>1.3.3</t>
+          <t>1.2.1.c</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr"/>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>2260 序列器 + 寄存器表</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr"/>
+      <c r="C22" s="7" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>3-bit / 偏心几何 (D8/D9)</t>
+        </is>
+      </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>配置广播一致; 寄存器表 pROM 初始化对</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>✅完成</t>
+          <t>棋盘/斜坡与 7020 同图; 转起来体像方向对</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>🔶进行中</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>自测</t>
+          <t>系统</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>ACG525</t>
+          <t>2047 屏 + 电机</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>仿真可</t>
+          <t>否</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>签名 1ED7F783/ACEED86D = 仿真</t>
-        </is>
-      </c>
-      <c r="M22" s="7" t="inlineStr"/>
+          <t>D8 寄存器级: 回读对、面 B 相位 = A+71 (142 片); frame_period 须亮屏才更新, 31590 待验</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>目视 + 电机</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>1.3.4</t>
+          <t>1.2.2</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr"/>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>tx 阵列 + ODDR 出线</t>
+          <t>PL lz4 三引擎 (M90)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr"/>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>mini-LVDS 出线逐比特</t>
+          <t>解压正确 + 并发不扰取片</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1934,12 +1942,12 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>ACG525</t>
+          <t>DR1M90</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>仿真可</t>
+          <t>否</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -1949,50 +1957,54 @@
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>链0 300M 过跳线 19 min 0 错</t>
-        </is>
-      </c>
-      <c r="M23" s="7" t="inlineStr"/>
+          <t>3000 帧全走 PL 0 回退, 71.7 ms/帧 (0.98 B/clk); ⚠ M90 上 CPU 解码 9.9 ms + 拷贝 14.5 ms ≈ 25 ms, CPU 反而快 3 倍</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>D10 改为 CPU 为主</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>1.3.5</t>
+          <t>1.2.3</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr"/>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>验证板配置 (60 扫 1串2)</t>
+          <t>上行发送 uplink_tx (→GW5A)</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr"/>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>桥片按验证板屏参数化: CASCADE=2、LINES=60、本屏链数、DCLK 166.67</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>13 lane 真帧 + 转发时钟, 800M / 1.0G; M90 位流</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>🔶进行中</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>自测</t>
+          <t>自测→合测</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>无 (仿真+综合); 上样板需 2260 样板</t>
+          <t>合测: DR1M90+ACG525 飞线 (换 0Ω 排阻, J2=1.8V)</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>综合/仿真已离线完成</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
@@ -2002,89 +2014,73 @@
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>现固件按目标板 24 链×1 颗×48 扫写</t>
+          <t>uplink_tx/m90: 800M/1.0G bin 出, pclk 余量 46%/26%; 仿真接 GW5A 真接收端逐字节 PASS (dr1v90 c73a5a7)</t>
         </is>
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
-          <t>★ 可先跑 (agent A)</t>
+          <t>D13/X2 上板</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>1.3.5.a</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr"/>
-      <c r="C25" s="7" t="inlineStr"/>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>参数化 + 仿真对拍</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>独立解码器逐像素; 级联第 2 颗语义 (09-21 台架结论)</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>自测</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="K25" s="7" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="L25" s="7" t="inlineStr"/>
-      <c r="M25" s="7" t="inlineStr"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>GW5A-25 · 桥片固件</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>上行接收 → 分发 → 2260 序列器 → tx 阵列; 两模式</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>🔶进行中</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="H25" s="5" t="inlineStr"/>
+      <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="5" t="inlineStr"/>
+      <c r="K25" s="5" t="inlineStr"/>
+      <c r="L25" s="5" t="inlineStr"/>
+      <c r="M25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>1.3.5.b</t>
+          <t>1.3.1</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr"/>
-      <c r="C26" s="7" t="inlineStr"/>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>DCLK 166.67 时序收敛</t>
-        </is>
-      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>上行接收 rtl_x8</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr"/>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>整桥 166.67 MHz 0 违例 (现 150)</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>IDES8 + 对齐 + deskew</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
@@ -2093,12 +2089,12 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>ACG525</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>仿真可</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
@@ -2108,85 +2104,93 @@
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>project_pov3d_trial_board_503_slices_60scan_ok</t>
-        </is>
-      </c>
-      <c r="M26" s="7" t="inlineStr"/>
+          <t>gw5a_loop 4lane@400M 硅上 0 错; bench 13 lane 片内</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="inlineStr">
+        <is>
+          <t>800M 长线待短绞线</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>1.3.5.c</t>
+          <t>1.3.2</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr"/>
-      <c r="C27" s="7" t="inlineStr"/>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>2260 样板出图 (D15)</t>
-        </is>
-      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>分发 + 帧门控</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr"/>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>已知图案; 1串2 写入</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>逐像素正确; 刷新不坏帧 (UL_DROP)</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>合测</t>
+          <t>自测</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>GW5A + 2260 样板</t>
+          <t>ACG525</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>仿真可</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="L27" s="7" t="inlineStr"/>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>gw5a_bench 1025 万帧 0 坏, 0 retrain</t>
+        </is>
+      </c>
       <c r="M27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>1.3.6</t>
+          <t>1.3.3</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr"/>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>压测模式</t>
+          <t>2260 序列器 + 寄存器表</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr"/>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>48 扫帧长 / 603 片 / 假 24 链满载, 误码可见</t>
-        </is>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>配置广播一致; 寄存器表 pROM 初始化对</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G28" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
@@ -2195,12 +2199,12 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>无 (仿真) / ACG525</t>
+          <t>ACG525</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>仿真可</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
@@ -2208,38 +2212,38 @@
           <t>是</t>
         </is>
       </c>
-      <c r="L28" s="7" t="inlineStr"/>
-      <c r="M28" s="7" t="inlineStr">
-        <is>
-          <t>D17</t>
-        </is>
-      </c>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>签名 1ED7F783/ACEED86D = 仿真</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>1.3.7</t>
+          <t>1.3.4</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr"/>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>真引脚 (转接板网表)</t>
+          <t>tx 阵列 + ODDR 出线</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr"/>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>按逐球引脚分配重排 IO_LOC, 出 bit</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>mini-LVDS 出线逐比特</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
@@ -2248,12 +2252,12 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>ACG525</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>仿真可</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -2263,40 +2267,36 @@
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>POV3D_GW5A转LED转接板_逐球引脚分配_2026-09-16</t>
-        </is>
-      </c>
-      <c r="M29" s="7" t="inlineStr">
-        <is>
-          <t>可先做</t>
-        </is>
-      </c>
+          <t>链0 300M 过跳线 19 min 0 错</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>1.3.8</t>
+          <t>1.3.5</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr"/>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>刷新不丢帧 (X3)</t>
+          <t>验证板配置 (60 扫 1串2)</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr"/>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>分块刷新, 帧号跳 0</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>每面 6 链×2 颗, 18 数据对 + 6 时钟对; 4,800 字槽/链/帧; DCLK 166.67; 4,296 fps</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>🔶进行中</t>
         </is>
       </c>
       <c r="G30" s="7" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>ACG525</t>
+          <t>上样板需 2260 样板</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
@@ -2320,40 +2320,40 @@
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>现每秒干净丢 1 帧</t>
+          <t>build_gw5a.sh 25S "" VALID; README 验证板 profile (dr1v90 f088f31)</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
-          <t>待定, 放 M3 后</t>
+          <t>1.3.5.c 上样板 (D15)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>1.3.9</t>
+          <t>1.3.5.a</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr"/>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>lane 47 单字错</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr"/>
+      <c r="C31" s="7" t="inlineStr"/>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>参数化 + 仿真对拍</t>
+        </is>
+      </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>判定量具问题还是桥问题</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>🔶进行中</t>
+          <t>独立解码器逐像素; 级联语义; 刷新压力档</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G31" s="7" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
@@ -2362,12 +2362,12 @@
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>ACG525</t>
+          <t>无</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -2377,85 +2377,89 @@
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>改量具后 1.3 h 0 错, 长跑中</t>
-        </is>
-      </c>
-      <c r="M31" s="7" t="inlineStr">
-        <is>
-          <t>读计数</t>
-        </is>
-      </c>
+          <t>5 真帧逐字全对 + VCRC; 每 3 帧刷新也无坏帧; 目标板回归逐行相同</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>1.3.10</t>
+          <t>1.3.5.b</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr"/>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>ACK 回读</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr"/>
+      <c r="C32" s="7" t="inlineStr"/>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>DCLK 166.67 时序收敛</t>
+        </is>
+      </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>2260 回包解析</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>⛔阻塞</t>
+          <t>整桥 166.67 MHz 0 违例</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G32" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>合测</t>
+          <t>自测</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>2260</t>
+          <t>无</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>project_icnd2260_ack_never_received</t>
-        </is>
-      </c>
-      <c r="M32" s="7" t="inlineStr"/>
+          <t>dclk 166.871 MHz, LUT 5179, BSRAM 48/56</t>
+        </is>
+      </c>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t>⚠ 4,296 fps 余量仅 0.2%, 可把 IDLE_CLK 64→32 换 0.6 µs (需上板确认)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>1.3.11</t>
+          <t>1.3.5.c</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr"/>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Flash 冷启动</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr"/>
-      <c r="E33" s="7" t="inlineStr"/>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>⏸跳过</t>
+      <c r="C33" s="7" t="inlineStr"/>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>2260 样板出图 (D15)</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>已知图案; 1串2 写入</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>⬜未开始</t>
         </is>
       </c>
       <c r="G33" s="7" t="n">
@@ -2463,80 +2467,100 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
+          <t>合测</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>GW5A + 2260 样板</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="inlineStr"/>
+      <c r="M33" s="7" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>1.3.6</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr"/>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>压测模式</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr"/>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>48 扫帧长 / 603 片 / 假 24 链满载, 误码可见</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
           <t>自测</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
-        <is>
-          <t>ACG525</t>
-        </is>
-      </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="K33" s="7" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="L33" s="7" t="inlineStr">
-        <is>
-          <t>用户定跳过 (Flash 内容不明)</t>
-        </is>
-      </c>
-      <c r="M33" s="7" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>1.4</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>PC · 上位机</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr"/>
-      <c r="D34" s="5" t="inlineStr"/>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>渲染/切片/体素表/推流</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>🔶进行中</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="H34" s="5" t="inlineStr"/>
-      <c r="I34" s="5" t="inlineStr"/>
-      <c r="J34" s="5" t="inlineStr"/>
-      <c r="K34" s="5" t="inlineStr"/>
-      <c r="L34" s="5" t="inlineStr"/>
-      <c r="M34" s="5" t="inlineStr"/>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>无 (仿真) / ACG525</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>10-12 GW5A_PROFILE_STRESS (dr1v90 977d694, 合入 feature/lvds-b2b efbab52): 正例 PASS 9,045 fps 0 错 FIFO 257/384; 注错 INJ-DETECTED 片上与 TB 一致; START_SLOTS 248; 25S 综合 BIT OK dclk 167.19 MHz TNS 0 LUT 6451</t>
+        </is>
+      </c>
+      <c r="M34" s="7" t="inlineStr">
+        <is>
+          <t>D17 上 ACG525 未做; 最差 setup +0.019 ns 在校验器</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.3.7</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr"/>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>2047 现役管线</t>
+          <t>真引脚 (转接板网表)</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr"/>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>7020 上已出体像</t>
+          <t>按逐球引脚分配重排 IO_LOC, 出 bit</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -2549,65 +2573,69 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>系统</t>
+          <t>自测</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>7020 台架</t>
+          <t>无</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>是</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>是</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>project_pov3d_dual_panel_volumetric_ok</t>
-        </is>
-      </c>
-      <c r="M35" s="7" t="inlineStr"/>
+          <t>10-12 数据源改 10-10 原理图 (09-16 分配已作废); 专用顶层 adapter/ + PINS=adapter (dr1v90 f0c85a2, 合入 efbab52); BIT OK dclk 193 / pclk 123 MHz TNS 0, 38 对差分核对通过; B5_B26 可作 PLL 参考</t>
+        </is>
+      </c>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>🔴 6 链首映射临时 (待新灯板原理图); 上行 lane 按契约 UL_D[k] 而非网名 TXPk; IDES8 复位 recovery −1.6 ns 为共用层原有问题; R176–R181/UL_CLK 100 MHz 待确认</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>1.4.2</t>
+          <t>1.3.12</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr"/>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>验证板口径推流</t>
+          <t>跨板接收时钟</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr"/>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>160×180, 358 片/圈 @12 rev/s; 体素表 (不传全切片)</t>
-        </is>
-      </c>
-      <c r="F36" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>PLL 参考 = DR1 转发时钟 (线速/8, 鉴相 ÷2); IODELAY + IDES8 + 扫眼 + 极性</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>自测</t>
+          <t>自测→合测</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>板上验证并入 D13</t>
         </is>
       </c>
       <c r="J36" s="7" t="inlineStr">
@@ -2622,117 +2650,145 @@
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
-          <t>wt-scatter VXT1 格式已有</t>
+          <t>仿真: 800M/1.0G +100 ppm 各 10 万 beat 0 错; ±300 ppm、PLL 相位扫参全过; 反例本地参考链路起不来, 2 ppm 下 7.4 万错 (dr1v90 419a60e)</t>
         </is>
       </c>
       <c r="M36" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>上板并入 D13</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>系统联调 (四门)</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr"/>
-      <c r="D37" s="5" t="inlineStr"/>
-      <c r="E37" s="5" t="inlineStr"/>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>1.3.13</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr"/>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>ACG525 上行接收工程 (X2)</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr"/>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>13 对 P6 + 转发时钟 P11-20, 后接出货桥核心 + vid_check; 板上 train → 等 S 行 done → go</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
         <is>
           <t>🔶进行中</t>
         </is>
       </c>
-      <c r="G37" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>系统</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr"/>
-      <c r="J37" s="5" t="inlineStr"/>
-      <c r="K37" s="5" t="inlineStr"/>
-      <c r="L37" s="5" t="inlineStr"/>
-      <c r="M37" s="5" t="inlineStr"/>
+      <c r="G37" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>合测</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>DR1M90 + ACG525 飞线 (FS03 换 0Ω, J2=1.8V)</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>构建已完成</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
+          <t>BIT OK pclk 127 / dclk 151.6 MHz; README gw5a_xboard/README.md</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>D13 上板</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>1.5.1</t>
+          <t>1.3.14</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr"/>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>M1 2047 双面全白</t>
+          <t>目标板帧间空闲 vs 链路看门狗</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr"/>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
-        </is>
-      </c>
-      <c r="F38" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>DR1 帧间空闲 5.3 µs 正好卡在 lane_align 掉锁看门狗 (5.12 µs) 边上, 降速即每帧重训练; 评估目标板默认开 UL_IDLE_OK</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G38" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>系统</t>
+          <t>自测</t>
         </is>
       </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>DR1M90 + 2047 屏</t>
+          <t>无</t>
         </is>
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="L38" s="7" t="inlineStr"/>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t>10-12 目标板默认 UL_IDLE_OK=1 (dr1v90 077d494, 合入 efbab52): 回归签名 1ED7F783/ACEED86D 与改前逐行同; 降速 250/113 µs 开 → retrain 0, 关 → 每帧重训练 (10/15 次); 25S 综合 152.49 MHz LUT 6077 (+32)</t>
+        </is>
+      </c>
       <c r="M38" s="7" t="inlineStr">
         <is>
-          <t>等屏 (焊接 ~2 h)</t>
+          <t>bench_top/xb_rx_top 显式传 0; xb_rx 建议下次 1.3.13 上机时改 1 并复测</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>1.5.2</t>
+          <t>1.3.8</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr"/>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>M2 推流体像</t>
+          <t>刷新不丢帧 (X3)</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr"/>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>D10, 10–12 fps 档</t>
+          <t>分块刷新, 帧号跳 0</t>
         </is>
       </c>
       <c r="F39" s="10" t="inlineStr">
@@ -2745,61 +2801,69 @@
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>系统</t>
+          <t>自测</t>
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>+ 电机 + WiFi</t>
+          <t>ACG525</t>
         </is>
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="L39" s="7" t="inlineStr"/>
-      <c r="M39" s="7" t="inlineStr"/>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L39" s="7" t="inlineStr">
+        <is>
+          <t>现每秒干净丢 1 帧</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t>待定, 放 M3 后</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>1.5.3</t>
+          <t>1.3.9</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr"/>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>M3 主控↔桥环回</t>
+          <t>lane 47 单字错</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr"/>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>D13, ≥3 min 零误码 (800M + 1.0G)</t>
-        </is>
-      </c>
-      <c r="F40" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>判定量具问题还是桥问题</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
         </is>
       </c>
       <c r="G40" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>合测</t>
+          <t>自测</t>
         </is>
       </c>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>DR1M90 + ACG525 + 飞线</t>
+          <t>ACG525</t>
         </is>
       </c>
       <c r="J40" s="7" t="inlineStr">
@@ -2809,33 +2873,41 @@
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="L40" s="7" t="inlineStr"/>
-      <c r="M40" s="7" t="inlineStr"/>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L40" s="7" t="inlineStr">
+        <is>
+          <t>10-12 结论: 量具问题, 桥无问题 —— 改量具后连续 47.9 h 15.6 亿帧 0 坏帧, 全 lane 3.45e15 bit 0 错 (BER 95% 上限 8.7e-16); 根因 vid_check 采样使能组合逻辑余量 +0.001 ns, 寄存一拍后消失</t>
+        </is>
+      </c>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>证明的是新量具这一版布局下桥 0 错</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>1.5.4</t>
+          <t>1.3.10</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr"/>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>M4 两模式 + 开机 + 远程</t>
+          <t>ACK 回读</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr"/>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
-        </is>
-      </c>
-      <c r="F41" s="10" t="inlineStr">
-        <is>
-          <t>⬜未开始</t>
+          <t>2260 回包解析</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>⛔阻塞</t>
         </is>
       </c>
       <c r="G41" s="7" t="n">
@@ -2843,12 +2915,12 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>系统</t>
+          <t>合测</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>全套</t>
+          <t>2260</t>
         </is>
       </c>
       <c r="J41" s="7" t="inlineStr">
@@ -2861,30 +2933,30 @@
           <t>否</t>
         </is>
       </c>
-      <c r="L41" s="7" t="inlineStr"/>
+      <c r="L41" s="7" t="inlineStr">
+        <is>
+          <t>project_icnd2260_ack_never_received</t>
+        </is>
+      </c>
       <c r="M41" s="7" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>1.5.5</t>
+          <t>1.3.11</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr"/>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>验证板整机上转子</t>
+          <t>Flash 冷启动</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr"/>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>新灯板 + 转接板 + 转子 + WPT</t>
-        </is>
-      </c>
-      <c r="F42" s="11" t="inlineStr">
-        <is>
-          <t>⛔阻塞</t>
+      <c r="E42" s="7" t="inlineStr"/>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>⏸跳过</t>
         </is>
       </c>
       <c r="G42" s="7" t="n">
@@ -2892,33 +2964,519 @@
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
+          <t>自测</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>ACG525</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>用户定跳过 (Flash 内容不明)</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>PC · 上位机</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>渲染/切片/体素表/推流</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>🔶进行中</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="5" t="inlineStr"/>
+      <c r="J43" s="5" t="inlineStr"/>
+      <c r="K43" s="5" t="inlineStr"/>
+      <c r="L43" s="5" t="inlineStr"/>
+      <c r="M43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>1.4.1</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr"/>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>2047 现役管线</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr"/>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>7020 上已出体像</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
           <t>系统</t>
         </is>
       </c>
-      <c r="I42" s="7" t="inlineStr">
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>7020 台架</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
+          <t>project_pov3d_dual_panel_volumetric_ok</t>
+        </is>
+      </c>
+      <c r="M44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>1.4.2</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr"/>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>验证板口径推流</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr"/>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>160×180, 358 片 @12 rev/s; 体素表 VXT1 (不传全切片), PVS1 flags=VOXTAB|LZ4</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>✅完成</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>自测</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L45" s="7" t="inlineStr">
+        <is>
+          <t>povstream --profile vb358; 10 帧×2 面×358 片 e2e 对拍 PASS; 最重真实内容 175 KB/帧 = 16.8 Mbps @12 fps (WiFi 159 余 9.4×)</t>
+        </is>
+      </c>
+      <c r="M45" s="7" t="inlineStr">
+        <is>
+          <t>板端接收/切片 → 1.1.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>系统联调 (四门)</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>🔶进行中</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr"/>
+      <c r="J46" s="5" t="inlineStr"/>
+      <c r="K46" s="5" t="inlineStr"/>
+      <c r="L46" s="5" t="inlineStr"/>
+      <c r="M46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>1.5.1</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr"/>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>M1 2047 双面全白</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr"/>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>⬜未开始</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>DR1M90 + 2047 屏</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K47" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L47" s="7" t="inlineStr"/>
+      <c r="M47" s="7" t="inlineStr">
+        <is>
+          <t>等屏 (焊接 ~2 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>1.5.2</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr"/>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>M2 推流体像</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr"/>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>D10, 10–12 fps 档</t>
+        </is>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>⬜未开始</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>+ 电机 + WiFi</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L48" s="7" t="inlineStr"/>
+      <c r="M48" s="7" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>1.5.3</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr"/>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>M3 主控↔桥环回</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr"/>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>D13, ≥3 min 零误码 (800M + 1.0G)</t>
+        </is>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>⬜未开始</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>合测</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>DR1M90 + ACG525 + 飞线</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K49" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L49" s="7" t="inlineStr"/>
+      <c r="M49" s="7" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>1.5.4</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr"/>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>M4 两模式 + 开机 + 远程</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr"/>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="F50" s="10" t="inlineStr">
+        <is>
+          <t>⬜未开始</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>全套</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L50" s="7" t="inlineStr"/>
+      <c r="M50" s="7" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>1.5.6</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr"/>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>转接板改版前提 (软件依赖的硬件项)</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr"/>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>UL_CLK 改回 B4_B33 (GCLK/PLL 脚); JTAG 加 2.5↔3.3V 转换 + 下载座; FPC 尾部 64~72 按契约重排</t>
+        </is>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>⬜未开始</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>硬件</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>转接板下一版</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>改板结论 09-18 必改项, 10-10 补注"上行前提 / 远程升级前提"; 规格书 v3 10-10 修订 (UL_CLK 线速/8)</t>
+        </is>
+      </c>
+      <c r="M51" s="7" t="inlineStr">
+        <is>
+          <t>硬件同事改板时必须落实</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>1.5.5</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr"/>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>验证板整机上转子</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr"/>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>新灯板 + 转接板 + 转子 + WPT</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>⛔阻塞</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="I52" s="7" t="inlineStr">
         <is>
           <t>硬件未回</t>
         </is>
       </c>
-      <c r="J42" s="7" t="inlineStr">
+      <c r="J52" s="7" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="K42" s="7" t="inlineStr">
+      <c r="K52" s="7" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="L42" s="7" t="inlineStr">
+      <c r="L52" s="7" t="inlineStr">
         <is>
           <t>不在 20 日计划内</t>
         </is>
       </c>
-      <c r="M42" s="7" t="inlineStr"/>
+      <c r="M52" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M42"/>
+  <autoFilter ref="A1:M52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2985,10 +3543,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>2</v>
@@ -3001,10 +3559,11 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1.1.4 pov_rxd 收流/解码/翻页
-1.1.6 开机自启
+          <t>1.1.6 开机自启 / 打包
 1.1.7 远程状态回传
-1.1.8 JTAG 给 GW5A 灌 SRAM</t>
+1.1.8 JTAG 给 GW5A 灌 SRAM
+1.1.10 板端体素→切片
+1.1.11 远程升级 (X4)</t>
         </is>
       </c>
     </row>
@@ -3018,13 +3577,13 @@
         <v>3</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
@@ -3043,16 +3602,16 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>4</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2</v>
@@ -3060,8 +3619,7 @@
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>1.3.5 验证板配置 (60 扫 1串2)
-1.3.6 压测模式
-1.3.7 真引脚 (转接板网表)
+1.3.13 ACG525 上行接收工程 (X2)
 1.3.8 刷新不丢帧 (X3)</t>
         </is>
       </c>
@@ -3076,22 +3634,18 @@
         <v>2</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>1.4.2 验证板口径推流</t>
-        </is>
-      </c>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3100,7 +3654,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>0</v>
@@ -3109,7 +3663,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>1</v>

</xml_diff>